<commit_message>
Drop empty CICE detail shells and refresh Asia-Pacific finals.
Filter CICE listings whose pages are placeholder 'nothing' content, then rebuild aea/provincial/asia_pacific exports.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/application list.xlsx
+++ b/application list.xlsx
@@ -53693,7 +53693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M57"/>
+  <dimension ref="A1:M52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -54107,12 +54107,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Business School</t>
+          <t>BAY AREA INTERNATIONAL BUSINESS SCHOOL</t>
         </is>
       </c>
       <c r="H10" s="13" t="inlineStr">
         <is>
-          <t>Business School</t>
+          <t>BAY AREA INTERNATIONAL BUSINESS SCHOOL</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -54122,7 +54122,7 @@
       </c>
       <c r="K10" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=96DC1B7F3204BD16</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=4AC7F281ECBD2BA4</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -54139,17 +54139,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Beijing Normal University</t>
+          <t>Capital University of Economics and Business</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BAY AREA INTERNATIONAL BUSINESS SCHOOL</t>
+          <t>International School of Economics and Management</t>
         </is>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
-          <t>BAY AREA INTERNATIONAL BUSINESS SCHOOL</t>
+          <t>International School of Economics and Management</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -54159,7 +54159,7 @@
       </c>
       <c r="K11" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=4AC7F281ECBD2BA4</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=230A8F8CAE8FB702</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -54176,17 +54176,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Capital University of Economics and Business</t>
+          <t>Dongbei University of Finance &amp; Economics</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>International School of Economics and Management</t>
+          <t>Institute for Advanced Economic Research</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2024-12-01</t>
         </is>
       </c>
       <c r="H12" s="13" t="inlineStr">
         <is>
-          <t>International School of Economics and Management</t>
+          <t>Institute for Advanced Economic Research</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -54196,7 +54201,7 @@
       </c>
       <c r="K12" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=230A8F8CAE8FB702</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=416DCA32DD657A3E</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -54213,22 +54218,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Dongbei University of Finance &amp; Economics</t>
+          <t>Donghua University</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Institute for Advanced Economic Research</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>2024-12-01</t>
+          <t>Glorious Sun School of Business and Management</t>
         </is>
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
-          <t>Institute for Advanced Economic Research</t>
+          <t>Glorious Sun School of Business and Management</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -54238,7 +54238,7 @@
       </c>
       <c r="K13" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=416DCA32DD657A3E</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=1CE68DDB85B84365</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -54255,17 +54255,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Donghua University</t>
+          <t>East China Normal University</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Glorious Sun School of Business and Management</t>
+          <t>School of Economics and Management</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="H14" s="13" t="inlineStr">
         <is>
-          <t>Glorious Sun School of Business and Management</t>
+          <t>School of Economics and Management</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -54275,7 +54280,7 @@
       </c>
       <c r="K14" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=1CE68DDB85B84365</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=02D0B642A4713897</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -54292,22 +54297,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>East China Normal University</t>
+          <t>Fudan University</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>School of Economics and Management</t>
+          <t>School of Economics</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="H15" s="13" t="inlineStr">
         <is>
-          <t>School of Economics and Management</t>
+          <t>School of Economics</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -54317,7 +54322,7 @@
       </c>
       <c r="K15" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=02D0B642A4713897</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=E968D280DD59D564</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -54339,17 +54344,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>School of Economics</t>
+          <t>School of Management</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>Rolling</t>
         </is>
       </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
-          <t>School of Economics</t>
+          <t>School of Management</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -54359,7 +54364,7 @@
       </c>
       <c r="K16" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=E968D280DD59D564</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=E153FEE8CC8E11B5</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -54381,17 +54386,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>School of Management</t>
+          <t>International School of Finance</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Rolling</t>
+          <t>2024-12-01</t>
         </is>
       </c>
       <c r="H17" s="13" t="inlineStr">
         <is>
-          <t>School of Management</t>
+          <t>International School of Finance</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -54401,7 +54406,7 @@
       </c>
       <c r="K17" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=E153FEE8CC8E11B5</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=1EB0900D191FE938</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -54418,22 +54423,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Fudan University</t>
+          <t>Harbin Institute of Technology</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>International School of Finance</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>2024-12-01</t>
+          <t>School of Management</t>
         </is>
       </c>
       <c r="H18" s="13" t="inlineStr">
         <is>
-          <t>International School of Finance</t>
+          <t>School of Management</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -54443,7 +54443,7 @@
       </c>
       <c r="K18" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=1EB0900D191FE938</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=3ED8A58471D2F80B</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -54460,17 +54460,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Harbin Institute of Technology</t>
+          <t>Huazhong University of Science and Technology</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>School of Management</t>
+          <t>School of Economics, Huazhong University of Science &amp; Technology</t>
         </is>
       </c>
       <c r="H19" s="13" t="inlineStr">
         <is>
-          <t>School of Management</t>
+          <t>School of Economics, Huazhong University of Science &amp; Technology</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>CV; Job Market Paper; Letters of Reference</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -54480,7 +54485,7 @@
       </c>
       <c r="K19" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=3ED8A58471D2F80B</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=A380FA8882023C78</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -54497,22 +54502,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Huazhong University of Science and Technology</t>
+          <t>Hunan University</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>School of Economics, Huazhong University of Science &amp; Technology</t>
+          <t>School of Economics and Trade</t>
         </is>
       </c>
       <c r="H20" s="13" t="inlineStr">
         <is>
-          <t>School of Economics, Huazhong University of Science &amp; Technology</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>CV; Job Market Paper; Letters of Reference</t>
+          <t>School of Economics and Trade</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -54522,7 +54522,7 @@
       </c>
       <c r="K20" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=A380FA8882023C78</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=38CE3CA2770AB83B</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -54539,17 +54539,22 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Hunan University</t>
+          <t>Jinan University</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>School of Economics and Trade</t>
+          <t>School of Economics(SOE)</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2023-11-30</t>
         </is>
       </c>
       <c r="H21" s="13" t="inlineStr">
         <is>
-          <t>School of Economics and Trade</t>
+          <t>School of Economics(SOE)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -54559,7 +54564,7 @@
       </c>
       <c r="K21" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=38CE3CA2770AB83B</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=071E9B3AC5A0F760</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -54576,22 +54581,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Jinan University</t>
+          <t>Lanzhou University of Finance and Economics</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>School of Economics(SOE)</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>2023-11-30</t>
+          <t>the Office of Personnel</t>
         </is>
       </c>
       <c r="H22" s="13" t="inlineStr">
         <is>
-          <t>School of Economics(SOE)</t>
+          <t>the Office of Personnel</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -54601,7 +54601,7 @@
       </c>
       <c r="K22" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=071E9B3AC5A0F760</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=003923B6EFE42FFF</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -54618,17 +54618,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Lanzhou University of Finance and Economics</t>
+          <t>Nanjing Agricultural University</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>the Office of Personnel</t>
+          <t>College of Finance</t>
         </is>
       </c>
       <c r="H23" s="13" t="inlineStr">
         <is>
-          <t>the Office of Personnel</t>
+          <t>College of Finance</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -54638,7 +54638,7 @@
       </c>
       <c r="K23" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=003923B6EFE42FFF</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=41CE1E8D1AE20F34</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -54655,17 +54655,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Nanjing Agricultural University</t>
+          <t>Nanjing University</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>College of Finance</t>
+          <t>Business School</t>
         </is>
       </c>
       <c r="H24" s="13" t="inlineStr">
         <is>
-          <t>College of Finance</t>
+          <t>Business School</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -54675,7 +54675,7 @@
       </c>
       <c r="K24" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=41CE1E8D1AE20F34</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=5EE87D5DE6734D4D</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -54692,17 +54692,22 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Nanjing University</t>
+          <t>Nankai University</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Business School</t>
+          <t>School of Economics</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2025-12-07</t>
         </is>
       </c>
       <c r="H25" s="13" t="inlineStr">
         <is>
-          <t>Business School</t>
+          <t>School of Economics</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -54712,7 +54717,7 @@
       </c>
       <c r="K25" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=5EE87D5DE6734D4D</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=FDC08442010B7BC2</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -54734,17 +54739,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>School of Economics</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>2025-12-07</t>
+          <t>School of Finance</t>
         </is>
       </c>
       <c r="H26" s="13" t="inlineStr">
         <is>
-          <t>School of Economics</t>
+          <t>School of Finance</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -54754,7 +54754,7 @@
       </c>
       <c r="K26" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=FDC08442010B7BC2</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=96728BEC2B0A48B6</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -54771,17 +54771,22 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Nankai University</t>
+          <t>Peking University</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>School of Finance</t>
+          <t>Guanghua School of Management</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Rolling</t>
         </is>
       </c>
       <c r="H27" s="13" t="inlineStr">
         <is>
-          <t>School of Finance</t>
+          <t>Guanghua School of Management</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -54791,7 +54796,7 @@
       </c>
       <c r="K27" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=96728BEC2B0A48B6</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=B2D1A3FBC0575542</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -54813,17 +54818,17 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Guanghua School of Management</t>
+          <t>Peking University HSBC Business School</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Rolling</t>
+          <t>2026-12-08</t>
         </is>
       </c>
       <c r="H28" s="13" t="inlineStr">
         <is>
-          <t>Guanghua School of Management</t>
+          <t>Peking University HSBC Business School</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -54833,7 +54838,7 @@
       </c>
       <c r="K28" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=B2D1A3FBC0575542</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=6AA44C52147BF1AA</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -54850,22 +54855,27 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Peking University</t>
+          <t>Renmin University of China</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Peking University HSBC Business School</t>
+          <t>School of Economics</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-12-08</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="H29" s="13" t="inlineStr">
         <is>
-          <t>Peking University HSBC Business School</t>
+          <t>School of Economics</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>CV; Job Market Paper; Letters of Reference</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -54875,7 +54885,7 @@
       </c>
       <c r="K29" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=6AA44C52147BF1AA</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=D7AB329AF0E6B516</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -54892,17 +54902,22 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Remin University</t>
+          <t>Renmin University of China</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>School of Applied Economics</t>
+          <t>School of Finance, Renmin University of China</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="H30" s="13" t="inlineStr">
         <is>
-          <t>School of Applied Economics</t>
+          <t>School of Finance, Renmin University of China</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -54912,7 +54927,7 @@
       </c>
       <c r="K30" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=680004BD3C688FB5</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=A2C98A6CF51DA6B8</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -54929,27 +54944,22 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Renmin University of China</t>
+          <t>Shanghai Institute for Mathematics and Interdisciplinary Sciences</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>School of Economics</t>
+          <t>The Shanghai Institute for Mathematics and Interdisciplinary Sciences</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-03-31</t>
         </is>
       </c>
       <c r="H31" s="13" t="inlineStr">
         <is>
-          <t>School of Economics</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>CV; Job Market Paper; Letters of Reference</t>
+          <t>The Shanghai Institute for Mathematics and Interdisciplinary Sciences</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -54959,7 +54969,7 @@
       </c>
       <c r="K31" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=D7AB329AF0E6B516</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=D6296C379B46AFF9</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -54976,22 +54986,22 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Renmin University of China</t>
+          <t>Shanghai Jiao Tong University</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>School of Finance, Renmin University of China</t>
+          <t>Antai College of Economics and Management</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2026-11-15</t>
         </is>
       </c>
       <c r="H32" s="13" t="inlineStr">
         <is>
-          <t>School of Finance, Renmin University of China</t>
+          <t>Antai College of Economics and Management</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -55001,7 +55011,7 @@
       </c>
       <c r="K32" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=A2C98A6CF51DA6B8</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=A718B6651C5FE241</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -55018,22 +55028,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Shanghai Institute for Mathematics and Interdisciplinary Sciences</t>
+          <t>Shanghai University of Finance and Economics</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>The Shanghai Institute for Mathematics and Interdisciplinary Sciences</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>2025-03-31</t>
+          <t>School of Economics</t>
         </is>
       </c>
       <c r="H33" s="13" t="inlineStr">
         <is>
-          <t>The Shanghai Institute for Mathematics and Interdisciplinary Sciences</t>
+          <t>School of Economics</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -55043,7 +55048,7 @@
       </c>
       <c r="K33" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=D6296C379B46AFF9</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=3E6981392FF08E75</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -55060,22 +55065,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Shanghai Jiao Tong University</t>
+          <t>Shanghai University of Finance Economics School</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Antai College of Economics and Management</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>2026-11-15</t>
+          <t>School of Digital Economy</t>
         </is>
       </c>
       <c r="H34" s="13" t="inlineStr">
         <is>
-          <t>Antai College of Economics and Management</t>
+          <t>School of Digital Economy</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -55085,7 +55085,7 @@
       </c>
       <c r="K34" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=A718B6651C5FE241</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=7E509CEAE1E65959</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -55102,17 +55102,22 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Shanghai University of Finance and Economics</t>
+          <t>Sichuan University</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>School of Economics</t>
+          <t>The School of Economics of Sichuan University</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2024-06-30</t>
         </is>
       </c>
       <c r="H35" s="13" t="inlineStr">
         <is>
-          <t>School of Economics</t>
+          <t>The School of Economics of Sichuan University</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -55122,7 +55127,7 @@
       </c>
       <c r="K35" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=3E6981392FF08E75</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=4D01E5935B5738A3</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -55139,17 +55144,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Shanghai University of Finance Economics School</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>School of Digital Economy</t>
+          <t>Southern University of Science and Technology</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2023-12-10</t>
         </is>
       </c>
       <c r="H36" s="13" t="inlineStr">
         <is>
-          <t>School of Digital Economy</t>
+          <t>Southern University of Science and Technology</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -55159,7 +55164,7 @@
       </c>
       <c r="K36" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=7E509CEAE1E65959</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=3EF86BA9413BD79E</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -55176,17 +55181,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Shanghai University of Finance and Economics</t>
+          <t>Southwestern University of Finance and Economics</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Dishui Lake Advanced Finance Institute</t>
+          <t>School of Economics</t>
         </is>
       </c>
       <c r="H37" s="13" t="inlineStr">
         <is>
-          <t>Dishui Lake Advanced Finance Institute</t>
+          <t>School of Economics</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -55196,7 +55201,7 @@
       </c>
       <c r="K37" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=5D5B5B1874A95B18</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=8F2A4E7B41A62BEC</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -55213,22 +55218,27 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Sichuan University</t>
+          <t>Southwestern University of Finance&amp;;Economics</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>The School of Economics of Sichuan University</t>
+          <t>Research Institute of Economics and Management</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2024-06-30</t>
+          <t>2023-12-01</t>
         </is>
       </c>
       <c r="H38" s="13" t="inlineStr">
         <is>
-          <t>The School of Economics of Sichuan University</t>
+          <t>Research Institute of Economics and Management</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>CV; Job Market Paper; Letters of Reference</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -55238,7 +55248,7 @@
       </c>
       <c r="K38" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=4D01E5935B5738A3</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=DB9471D924F0FD44</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -55255,17 +55265,22 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Southern University of Science and Technology</t>
+          <t>Sun Yat-sen University</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Lingnan College</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2023-12-10</t>
+          <t>2023-05-12</t>
         </is>
       </c>
       <c r="H39" s="13" t="inlineStr">
         <is>
-          <t>Southern University of Science and Technology</t>
+          <t>Lingnan College</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -55275,7 +55290,7 @@
       </c>
       <c r="K39" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=3EF86BA9413BD79E</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=73CF283104D9C7BB</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -55292,17 +55307,22 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Southwestern University of Finance and Economics</t>
+          <t>The Chinese University of Hong Kong</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>School of Economics</t>
+          <t>Department of Economics</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2024-11-30</t>
         </is>
       </c>
       <c r="H40" s="13" t="inlineStr">
         <is>
-          <t>School of Economics</t>
+          <t>Department of Economics</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -55312,7 +55332,7 @@
       </c>
       <c r="K40" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=8F2A4E7B41A62BEC</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=0204A4EECEEA66C1</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -55329,27 +55349,22 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Southwestern University of Finance&amp;;Economics</t>
+          <t>Tianjin University</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Research Institute of Economics and Management</t>
+          <t>Ma Yinchu School of Economics</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2023-12-01</t>
+          <t>2023-11-15</t>
         </is>
       </c>
       <c r="H41" s="13" t="inlineStr">
         <is>
-          <t>Research Institute of Economics and Management</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>CV; Job Market Paper; Letters of Reference</t>
+          <t>Ma Yinchu School of Economics</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -55359,7 +55374,7 @@
       </c>
       <c r="K41" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=DB9471D924F0FD44</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=3514AA8724F3F9F8</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -55376,22 +55391,22 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Sun Yat-sen University</t>
+          <t>Tsinghua University</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Lingnan College</t>
+          <t>School of Economics and Management</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2023-05-12</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="H42" s="13" t="inlineStr">
         <is>
-          <t>Lingnan College</t>
+          <t>School of Economics and Management</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -55401,7 +55416,7 @@
       </c>
       <c r="K42" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=73CF283104D9C7BB</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=EB34146E1220A115</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -55418,22 +55433,17 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>The Chinese University of Hong Kong</t>
+          <t>Tsinghua University</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Department of Economics</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>2024-11-30</t>
+          <t>Center for International Finance and Economics Research</t>
         </is>
       </c>
       <c r="H43" s="13" t="inlineStr">
         <is>
-          <t>Department of Economics</t>
+          <t>Center for International Finance and Economics Research</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -55443,7 +55453,7 @@
       </c>
       <c r="K43" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=0204A4EECEEA66C1</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=6A1E66715A3A82D9</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -55460,22 +55470,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Tianjin University</t>
+          <t>University of Electronic Science and Technology of China</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Ma Yinchu School of Economics</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>2023-11-15</t>
+          <t>School of Management and Economics</t>
         </is>
       </c>
       <c r="H44" s="13" t="inlineStr">
         <is>
-          <t>Ma Yinchu School of Economics</t>
+          <t>School of Management and Economics</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -55485,7 +55490,7 @@
       </c>
       <c r="K44" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=3514AA8724F3F9F8</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=390B333672086D05</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -55502,17 +55507,17 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Tongji University</t>
+          <t>University of Science and Technology of China</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>nothing</t>
+          <t>School of Management</t>
         </is>
       </c>
       <c r="H45" s="13" t="inlineStr">
         <is>
-          <t>nothing</t>
+          <t>School of Management</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -55522,7 +55527,7 @@
       </c>
       <c r="K45" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=41EFAE6DC817CCD8</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=6CAF00207D46BD36</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -55539,17 +55544,17 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Tsinghua University</t>
+          <t>University of Science and Technology of China</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>School of Social Sciences</t>
+          <t>Institute of International Finance</t>
         </is>
       </c>
       <c r="H46" s="13" t="inlineStr">
         <is>
-          <t>School of Social Sciences</t>
+          <t>Institute of International Finance</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -55559,7 +55564,7 @@
       </c>
       <c r="K46" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=48673CE5E9319FD6</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=612A2FEECB1FB3D7</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
@@ -55576,7 +55581,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Tsinghua University</t>
+          <t>Wuhan University</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -55586,7 +55591,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2023-11-30</t>
         </is>
       </c>
       <c r="H47" s="13" t="inlineStr">
@@ -55601,7 +55606,7 @@
       </c>
       <c r="K47" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=EB34146E1220A115</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=A2DDB669D0484F72</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -55618,17 +55623,17 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Tsinghua University</t>
+          <t>Xi%u2019an Jiaotong University</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Center for International Finance and Economics Research</t>
+          <t>School of Economics and Finance</t>
         </is>
       </c>
       <c r="H48" s="13" t="inlineStr">
         <is>
-          <t>Center for International Finance and Economics Research</t>
+          <t>School of Economics and Finance</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -55638,7 +55643,7 @@
       </c>
       <c r="K48" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=6A1E66715A3A82D9</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=C3A72C51D391769E</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -55655,17 +55660,17 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>University of Electronic Science and Technology of China</t>
+          <t>Xi%u2019an Jiaotong-Liverpool University</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>School of Management and Economics</t>
+          <t>International Business School Suzhou (IBSS), Department of Economics</t>
         </is>
       </c>
       <c r="H49" s="13" t="inlineStr">
         <is>
-          <t>School of Management and Economics</t>
+          <t>International Business School Suzhou (IBSS), Department of Economics</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -55675,7 +55680,7 @@
       </c>
       <c r="K49" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=390B333672086D05</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=038CBF83FD61166B</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -55692,17 +55697,22 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>University of Science and Technology of China</t>
+          <t>Zhejiang University</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>School of Management</t>
+          <t>School of Economics</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="H50" s="13" t="inlineStr">
         <is>
-          <t>School of Management</t>
+          <t>School of Economics</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -55712,7 +55722,7 @@
       </c>
       <c r="K50" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=6CAF00207D46BD36</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=7D928B7B1C35099A</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
@@ -55729,17 +55739,17 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>University of Science and Technology of China</t>
+          <t>Zhejiang University</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Institute of International Finance</t>
+          <t>International Business School</t>
         </is>
       </c>
       <c r="H51" s="13" t="inlineStr">
         <is>
-          <t>Institute of International Finance</t>
+          <t>International Business School</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -55749,7 +55759,7 @@
       </c>
       <c r="K51" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=612A2FEECB1FB3D7</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=AB6EF80CCC4E40B3</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
@@ -55766,22 +55776,17 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Wuhan University</t>
+          <t>Zhongnan Unviersity of Economics and Law</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>School of Economics and Management</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>2023-11-30</t>
+          <t>School of Finance</t>
         </is>
       </c>
       <c r="H52" s="13" t="inlineStr">
         <is>
-          <t>School of Economics and Management</t>
+          <t>School of Finance</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -55791,200 +55796,10 @@
       </c>
       <c r="K52" s="13" t="inlineStr">
         <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=A2DDB669D0484F72</t>
+          <t>http://www.cicecon.org.cn/careers/detail.html?k=2FC3B168FE2DBD23</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
-        <is>
-          <t>Faculty</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>China</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Xi%u2019an Jiaotong University</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>School of Economics and Finance</t>
-        </is>
-      </c>
-      <c r="H53" s="13" t="inlineStr">
-        <is>
-          <t>School of Economics and Finance</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>CICE</t>
-        </is>
-      </c>
-      <c r="K53" s="13" t="inlineStr">
-        <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=C3A72C51D391769E</t>
-        </is>
-      </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>Faculty</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>China</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Xi%u2019an Jiaotong-Liverpool University</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>International Business School Suzhou (IBSS), Department of Economics</t>
-        </is>
-      </c>
-      <c r="H54" s="13" t="inlineStr">
-        <is>
-          <t>International Business School Suzhou (IBSS), Department of Economics</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>CICE</t>
-        </is>
-      </c>
-      <c r="K54" s="13" t="inlineStr">
-        <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=038CBF83FD61166B</t>
-        </is>
-      </c>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t>Faculty</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>China</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Zhejiang University</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>School of Economics</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>2025-11-28</t>
-        </is>
-      </c>
-      <c r="H55" s="13" t="inlineStr">
-        <is>
-          <t>School of Economics</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>CICE</t>
-        </is>
-      </c>
-      <c r="K55" s="13" t="inlineStr">
-        <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=7D928B7B1C35099A</t>
-        </is>
-      </c>
-      <c r="M55" t="inlineStr">
-        <is>
-          <t>Faculty</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>China</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Zhejiang University</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>International Business School</t>
-        </is>
-      </c>
-      <c r="H56" s="13" t="inlineStr">
-        <is>
-          <t>International Business School</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>CICE</t>
-        </is>
-      </c>
-      <c r="K56" s="13" t="inlineStr">
-        <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=AB6EF80CCC4E40B3</t>
-        </is>
-      </c>
-      <c r="M56" t="inlineStr">
-        <is>
-          <t>Faculty</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>China</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>Zhongnan Unviersity of Economics and Law</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>School of Finance</t>
-        </is>
-      </c>
-      <c r="H57" s="13" t="inlineStr">
-        <is>
-          <t>School of Finance</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>CICE</t>
-        </is>
-      </c>
-      <c r="K57" s="13" t="inlineStr">
-        <is>
-          <t>http://www.cicecon.org.cn/careers/detail.html?k=2FC3B168FE2DBD23</t>
-        </is>
-      </c>
-      <c r="M57" t="inlineStr">
         <is>
           <t>Faculty</t>
         </is>
@@ -56094,16 +55909,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K51" r:id="rId100"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId101"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K52" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K53" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K54" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K55" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K56" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K57" r:id="rId112"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>